<commit_message>
add patient features added
</commit_message>
<xml_diff>
--- a/testData/testData.xlsx
+++ b/testData/testData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayau\OneDrive\Desktop\Playwright\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\Projects\Team6_Playwright_Warriors_Dietician_Hackathon\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D99BB85-DF71-46FB-978B-C74CD08CC052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B8EF124-15F4-4DB7-BDA1-8DC1DEDFC005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA13B433-7DF9-48CA-B533-07C4F7CAE878}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA13B433-7DF9-48CA-B533-07C4F7CAE878}"/>
   </bookViews>
   <sheets>
-    <sheet name="editPatient" sheetId="1" r:id="rId1"/>
+    <sheet name="addPatient" sheetId="2" r:id="rId1"/>
+    <sheet name="editPatient" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="133">
   <si>
     <t>Scenario</t>
   </si>
@@ -277,13 +278,169 @@
   </si>
   <si>
     <t>Please enter a valid DP value</t>
+  </si>
+  <si>
+    <t>scenarioName</t>
+  </si>
+  <si>
+    <t>ContactNumber</t>
+  </si>
+  <si>
+    <t>Allergy</t>
+  </si>
+  <si>
+    <t>CuisineCategory</t>
+  </si>
+  <si>
+    <t>ExpectedResult</t>
+  </si>
+  <si>
+    <t>FN_Numeric</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>arulkumar01@test.com</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>Vegetarian</t>
+  </si>
+  <si>
+    <t>Punjabi</t>
+  </si>
+  <si>
+    <t>01/12/2000</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>98.6</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>Patient first name accepts only alphabets</t>
+  </si>
+  <si>
+    <t>FN_SpecialChar</t>
+  </si>
+  <si>
+    <t>@@@@</t>
+  </si>
+  <si>
+    <t>FN_Empty</t>
+  </si>
+  <si>
+    <t>Patient first name is required</t>
+  </si>
+  <si>
+    <t>LN_Numeric</t>
+  </si>
+  <si>
+    <t>Arul</t>
+  </si>
+  <si>
+    <t>Patient last name accepts only alphabets</t>
+  </si>
+  <si>
+    <t>Email_NoAt</t>
+  </si>
+  <si>
+    <t>Please enter valid email address</t>
+  </si>
+  <si>
+    <t>Email_Exists</t>
+  </si>
+  <si>
+    <t>Email address already exists</t>
+  </si>
+  <si>
+    <t>Contact_Alpha</t>
+  </si>
+  <si>
+    <t>abcd</t>
+  </si>
+  <si>
+    <t>Please enter valid contact number</t>
+  </si>
+  <si>
+    <t>Contact_Short</t>
+  </si>
+  <si>
+    <t>Allergy_Empty</t>
+  </si>
+  <si>
+    <t>Allergy information is required</t>
+  </si>
+  <si>
+    <t>DOB_Empty</t>
+  </si>
+  <si>
+    <t>Date of Birth is required</t>
+  </si>
+  <si>
+    <t>Weight_Special</t>
+  </si>
+  <si>
+    <t>@@@</t>
+  </si>
+  <si>
+    <t>Please enter valid weight</t>
+  </si>
+  <si>
+    <t>Height_Alpha</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>Please enter valid height</t>
+  </si>
+  <si>
+    <t>Temp_Alpha</t>
+  </si>
+  <si>
+    <t>Please enter valid temperature</t>
+  </si>
+  <si>
+    <t>SPDP_Alpha</t>
+  </si>
+  <si>
+    <t>xyz</t>
+  </si>
+  <si>
+    <t>Please enter valid SP,DP</t>
+  </si>
+  <si>
+    <t>All_Valid</t>
+  </si>
+  <si>
+    <t>Patient successfully created</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +452,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -355,16 +520,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -380,8 +544,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -398,9 +565,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -438,7 +605,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -544,7 +711,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -686,30 +853,793 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D59B3C-7078-4C9A-9C82-689CF20841C9}">
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N3" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M5" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N5" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6" s="12">
+        <v>12345</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O10" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N11" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O11" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="N15" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="N16" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="O16" s="11" t="s">
+        <v>132</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{8713DEC4-7F40-4484-BB72-387B2BD1E735}"/>
+    <hyperlink ref="D3:D16" r:id="rId2" display="arulkumar01@test.com" xr:uid="{E5AEE2D8-7549-42A3-A330-E0BC9A4844FB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{183ED1C6-A774-4CA5-97B7-F76D87ACF366}">
   <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.140625" style="12"/>
-    <col min="12" max="12" width="12.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.140625" style="12"/>
-    <col min="15" max="15" width="62.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.109375" style="10"/>
+    <col min="12" max="12" width="12.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.109375" style="10"/>
+    <col min="15" max="15" width="62.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -737,45 +1667,45 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="8"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="6"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -789,16 +1719,16 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
       <c r="O3" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -812,16 +1742,16 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
       <c r="O4" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
@@ -835,16 +1765,16 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
       <c r="O5" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
@@ -858,22 +1788,22 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
       <c r="O6" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="5" t="s">
+      <c r="D7" t="s">
         <v>29</v>
       </c>
       <c r="E7" s="3"/>
@@ -881,16 +1811,16 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
       <c r="O7" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -904,16 +1834,16 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
       <c r="O8" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -925,16 +1855,16 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
       <c r="O9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -946,16 +1876,16 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
       <c r="O10" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -969,16 +1899,16 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
       <c r="O11" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
@@ -992,17 +1922,17 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
       <c r="O12" s="3" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B13" s="3"/>
@@ -1015,17 +1945,17 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="6" t="s">
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B14" s="3"/>
@@ -1036,17 +1966,17 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
       <c r="O14" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -1059,17 +1989,17 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
       <c r="O15" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="3"/>
@@ -1082,22 +2012,22 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
       <c r="O16" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
-      <c r="D17" s="5" t="s">
+      <c r="D17" t="s">
         <v>41</v>
       </c>
       <c r="E17" s="3"/>
@@ -1105,17 +2035,17 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
       <c r="O17" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B18" s="3"/>
@@ -1128,36 +2058,36 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
       <c r="O18" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="8"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="6"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B20" s="3"/>
@@ -1168,19 +2098,19 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
-      <c r="J20" s="11">
+      <c r="J20" s="9">
         <v>154</v>
       </c>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
       <c r="O20" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>53</v>
       </c>
       <c r="B21" s="3"/>
@@ -1191,19 +2121,19 @@
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
       <c r="O21" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B22" s="3"/>
@@ -1214,19 +2144,19 @@
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="11" t="s">
+      <c r="J22" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
       <c r="O22" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B23" s="3"/>
@@ -1237,19 +2167,19 @@
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11">
+      <c r="J23" s="9"/>
+      <c r="K23" s="9">
         <v>6</v>
       </c>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
       <c r="O23" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
         <v>56</v>
       </c>
       <c r="B24" s="3"/>
@@ -1260,19 +2190,19 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11" t="s">
+      <c r="J24" s="9"/>
+      <c r="K24" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
       <c r="O24" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B25" s="3"/>
@@ -1283,19 +2213,19 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11" t="s">
+      <c r="J25" s="9"/>
+      <c r="K25" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
       <c r="O25" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>58</v>
       </c>
       <c r="B26" s="3"/>
@@ -1306,19 +2236,19 @@
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11">
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9">
         <v>97</v>
       </c>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
       <c r="O26" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>59</v>
       </c>
       <c r="B27" s="3"/>
@@ -1329,19 +2259,19 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11" t="s">
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
       <c r="O27" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>60</v>
       </c>
       <c r="B28" s="3"/>
@@ -1352,19 +2282,19 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11" t="s">
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
       <c r="O28" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>61</v>
       </c>
       <c r="B29" s="3"/>
@@ -1375,19 +2305,19 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11">
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9">
         <v>120</v>
       </c>
-      <c r="N29" s="11"/>
+      <c r="N29" s="9"/>
       <c r="O29" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B30" s="3"/>
@@ -1398,19 +2328,19 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11" t="s">
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="N30" s="11"/>
+      <c r="N30" s="9"/>
       <c r="O30" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>63</v>
       </c>
       <c r="B31" s="3"/>
@@ -1421,19 +2351,19 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11" t="s">
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9"/>
+      <c r="M31" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="N31" s="11"/>
+      <c r="N31" s="9"/>
       <c r="O31" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
         <v>64</v>
       </c>
       <c r="B32" s="3"/>
@@ -1444,19 +2374,19 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11">
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9">
         <v>75</v>
       </c>
       <c r="O32" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B33" s="3"/>
@@ -1467,19 +2397,19 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11" t="s">
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9" t="s">
         <v>74</v>
       </c>
       <c r="O33" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B34" s="3"/>
@@ -1490,19 +2420,19 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11" t="s">
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9" t="s">
         <v>73</v>
       </c>
       <c r="O34" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>67</v>
       </c>
       <c r="B35" s="3"/>
@@ -1513,13 +2443,13 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11">
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9">
         <v>123</v>
       </c>
-      <c r="N35" s="11">
+      <c r="N35" s="9">
         <v>73</v>
       </c>
       <c r="O35" s="3" t="s">

</xml_diff>